<commit_message>
Added Requirements and Test Reports
</commit_message>
<xml_diff>
--- a/Requirements/ASSET_SMART_Requirements_V1.03.xlsx
+++ b/Requirements/ASSET_SMART_Requirements_V1.03.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="504">
   <si>
     <t>SENSEL TELEMATICS PVT LTD</t>
   </si>
@@ -120,6 +120,9 @@
   </si>
   <si>
     <t xml:space="preserve">The device shall detect digital IO pin state changes to initiate wake-up from Sleep mode </t>
+  </si>
+  <si>
+    <t>AST_T5</t>
   </si>
   <si>
     <t>AST_R6</t>
@@ -1232,7 +1235,7 @@
     <t>AST_T118</t>
   </si>
   <si>
-    <t>AST_100</t>
+    <t>AST_R100</t>
   </si>
   <si>
     <t>Smart Charging</t>
@@ -1244,7 +1247,7 @@
     <t>AST_T119</t>
   </si>
   <si>
-    <t>AST_101</t>
+    <t>AST_R101</t>
   </si>
   <si>
     <t>10  mins updation while Charging</t>
@@ -1256,7 +1259,7 @@
     <t>AST_T120</t>
   </si>
   <si>
-    <t>AST_102</t>
+    <t>AST_R102</t>
   </si>
   <si>
     <t>Charger IC Reset</t>
@@ -1268,7 +1271,7 @@
     <t>AST_T121</t>
   </si>
   <si>
-    <t>AST_103</t>
+    <t>AST_R103</t>
   </si>
   <si>
     <t>SIM FAIL Case</t>
@@ -1280,7 +1283,7 @@
     <t>AST_T122</t>
   </si>
   <si>
-    <t>AST_104</t>
+    <t>AST_R104</t>
   </si>
   <si>
     <t>External Hardware Watchdog Pulse</t>
@@ -1289,7 +1292,10 @@
     <t>The device shall output a hardware resetter pulse(CTR_WDG_PULSE) during boot initialization to reset and feed the external hardware supervisor IC.</t>
   </si>
   <si>
-    <t>AST_105</t>
+    <t>AST_T123</t>
+  </si>
+  <si>
+    <t>AST_R105</t>
   </si>
   <si>
     <t xml:space="preserve">Resetter </t>
@@ -1298,7 +1304,10 @@
     <t>The device should reset as per configured timing incase of hang.</t>
   </si>
   <si>
-    <t>AST_106</t>
+    <t>AST_T124</t>
+  </si>
+  <si>
+    <t>AST_R106</t>
   </si>
   <si>
     <t>Hardware Reset Source Logging</t>
@@ -1307,7 +1316,10 @@
     <t>The device shall detect and differentiate boot reset sources (external watchdog pin, internal IWDG watchdog, software reset, NRST pin) and log failure causes into system diagnostic flags.</t>
   </si>
   <si>
-    <t>AST_107</t>
+    <t>AST_T125</t>
+  </si>
+  <si>
+    <t>AST_R107</t>
   </si>
   <si>
     <t>SPI Serial Flash Auto-Formatting</t>
@@ -1316,7 +1328,10 @@
     <t>Upon first boot or detection of unformatted flash memory, the device shall automatically initialize, unlock block protection, and format serial SPI flash sectors for data logging and chip erase in case of config reset.</t>
   </si>
   <si>
-    <t>AST_108</t>
+    <t>AST_T126</t>
+  </si>
+  <si>
+    <t>AST_R108</t>
   </si>
   <si>
     <t>Dynamic UART Baud Rate Fallback</t>
@@ -1325,7 +1340,10 @@
     <t>The device shall monitor modem and GPS communication flags (GSM_FLAG_ADDR, GPS_FLAG_ADDR) and automatically adjust or fallback UART baud rates to 9600 baud if communication instability is detected.</t>
   </si>
   <si>
-    <t>AST_109</t>
+    <t>AST_T127</t>
+  </si>
+  <si>
+    <t>AST_R109</t>
   </si>
   <si>
     <t>GPS Stationary Jaggies Filter</t>
@@ -1334,7 +1352,10 @@
     <t>The device shall execute a position jitter filtering algorithm to filter out false stationary movement drift (jaggies) when the asset is stationary before storing or transmitting coordinates.</t>
   </si>
   <si>
-    <t>AST_110</t>
+    <t>AST_T128</t>
+  </si>
+  <si>
+    <t>AST_R110</t>
   </si>
   <si>
     <t>Cellular Tower (LAC / Cell ID) Positioning</t>
@@ -1343,7 +1364,10 @@
     <t>The device shall extract Location Area Code (LAC) and Cell ID (CI) from the cellular network to include cell tower telemetry in packets for network-based location triangulation when GPS fix is unavailable.</t>
   </si>
   <si>
-    <t>AST_111</t>
+    <t>AST_T129</t>
+  </si>
+  <si>
+    <t>AST_R111</t>
   </si>
   <si>
     <t>Dynamic Thermal Charging Protection</t>
@@ -1352,7 +1376,10 @@
     <t>The device shall continuously monitor battery thermistor temperature and battery voltage to dynamically toggle the charging control enable pin (CHR_EN) to prevent charging under high thermal conditions.</t>
   </si>
   <si>
-    <t>AST_112</t>
+    <t>AST_T130</t>
+  </si>
+  <si>
+    <t>AST_R112</t>
   </si>
   <si>
     <t>Dual Hardware Tamper Interfaces</t>
@@ -1361,7 +1388,10 @@
     <t>The device shall support dual hardware tamper detection interrupts: Tamper 1 for accelerometer orientation tamper (CTR_ACC_INT1) and Tamper 2 for magnetic reed switch / enclosure breach (CTR_TAMP_SW1).</t>
   </si>
   <si>
-    <t>AST_113</t>
+    <t>AST_T131</t>
+  </si>
+  <si>
+    <t>AST_R113</t>
   </si>
   <si>
     <t>High G-Force Impact Alert Detection</t>
@@ -1370,7 +1400,10 @@
     <t>The device shall monitor 3-axis accelerometer data for sudden G-force shock spikes above configured thresholds, set an impact event flag in telemetry packets, and clear impact registers post-dispatch.</t>
   </si>
   <si>
-    <t>AST_114</t>
+    <t>AST_T132</t>
+  </si>
+  <si>
+    <t>AST_R114</t>
   </si>
   <si>
     <t>Failed Upload Packet Flash Intercept</t>
@@ -1379,7 +1412,10 @@
     <t>In the event of a GPRS connection failure during live transmission, the device shall automatically intercept and queue unsent telemetry packets into external serial flash using a FIFO circular buffer.</t>
   </si>
   <si>
-    <t>AST_115</t>
+    <t>AST_T133</t>
+  </si>
+  <si>
+    <t>AST_R115</t>
   </si>
   <si>
     <t>Active State Safety Timeout Limit</t>
@@ -1388,7 +1424,10 @@
     <t>The device shall run a safety timeout watchdog during active wakeup cycles to enforce a maximum allowable active execution window and force low-power sleep if operations fail to finish.</t>
   </si>
   <si>
-    <t>AST_116</t>
+    <t>AST_T134</t>
+  </si>
+  <si>
+    <t>AST_R116</t>
   </si>
   <si>
     <t>Bluetooth / BLE Peripheral Beacon Scanning</t>
@@ -1397,7 +1436,10 @@
     <t>The device shall support Bluetooth/BLE peripheral scanning to detect nearby BLE beacons, parse BLE packet length, and extract beacon MAC IDs and RSSI values.</t>
   </si>
   <si>
-    <t>AST_117</t>
+    <t>AST_T135</t>
+  </si>
+  <si>
+    <t>AST_R117</t>
   </si>
   <si>
     <t>System Operating Current Monitoring</t>
@@ -1406,7 +1448,10 @@
     <t>The device shall interface with current sensor ADCs to sample operating current consumption during active tasks and optimize power management routines.</t>
   </si>
   <si>
-    <t>AST_118</t>
+    <t>AST_T136</t>
+  </si>
+  <si>
+    <t>AST_R118</t>
   </si>
   <si>
     <t>Cellular Signal (CSQ) &amp; Network Operator Check</t>
@@ -1415,7 +1460,10 @@
     <t>The device shall query cellular signal quality (CSQ/RSSI) and Network Operator registration status (COPS) to evaluate link viability prior to data transmission.</t>
   </si>
   <si>
-    <t>AST_119</t>
+    <t>AST_T137</t>
+  </si>
+  <si>
+    <t>AST_R119</t>
   </si>
   <si>
     <t>NMEA Satellite Fix Quality &amp; HDOP Parsing</t>
@@ -1424,7 +1472,10 @@
     <t>The device shall parse NMEA GPRMC and GPGGA sentences to extract satellite count in view, Horizontal Dilution of Precision (HDOP), altitude, and fix status for telemetry packets.</t>
   </si>
   <si>
-    <t>AST_120</t>
+    <t>AST_T138</t>
+  </si>
+  <si>
+    <t>AST_R120</t>
   </si>
   <si>
     <t>RTC Time Synchronization via GPS/GSM</t>
@@ -1433,13 +1484,19 @@
     <t>The device shall extract UTC timestamp data from valid GPS NMEA fixes or GSM network time to automatically synchronize and calibrate the internal RTC clock.</t>
   </si>
   <si>
-    <t>AST_121</t>
+    <t>AST_T139</t>
+  </si>
+  <si>
+    <t>AST_R121</t>
   </si>
   <si>
     <t>Packet Frame XOR / CRC Checksum Validation</t>
   </si>
   <si>
     <t>The device shall compute multi-byte XOR/CRC checksums for outgoing packet frames and validate incoming server response frames before executing commands.</t>
+  </si>
+  <si>
+    <t>AST_T140</t>
   </si>
   <si>
     <t>Revision History :</t>
@@ -1583,6 +1640,12 @@
     </font>
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -1593,12 +1656,6 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -2696,7 +2753,7 @@
     <xf numFmtId="10" fontId="39" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="36" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2766,12 +2823,12 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2790,41 +2847,32 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="184" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="184" fontId="11" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3419,7 +3467,9 @@
         <v>30</v>
       </c>
       <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
+      <c r="F14" s="31" t="s">
+        <v>31</v>
+      </c>
       <c r="G14" s="26"/>
       <c r="H14" s="26"/>
       <c r="I14" s="26"/>
@@ -3427,17 +3477,17 @@
     <row r="15" ht="60" customHeight="1" spans="1:9">
       <c r="A15" s="23"/>
       <c r="B15" s="27" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E15" s="28"/>
       <c r="F15" s="29" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G15" s="26"/>
       <c r="H15" s="26"/>
@@ -3446,17 +3496,17 @@
     <row r="16" ht="30" customHeight="1" spans="1:9">
       <c r="A16" s="23"/>
       <c r="B16" s="27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="31" t="s">
         <v>37</v>
+      </c>
+      <c r="D16" s="32" t="s">
+        <v>38</v>
       </c>
       <c r="E16" s="28"/>
       <c r="F16" s="29" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G16" s="26"/>
       <c r="H16" s="26"/>
@@ -3465,17 +3515,17 @@
     <row r="17" ht="60" customHeight="1" spans="1:9">
       <c r="A17" s="23"/>
       <c r="B17" s="27" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D17" s="27" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E17" s="28"/>
       <c r="F17" s="29" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G17" s="26"/>
       <c r="H17" s="26"/>
@@ -3484,17 +3534,17 @@
     <row r="18" ht="30" customHeight="1" spans="1:9">
       <c r="A18" s="23"/>
       <c r="B18" s="27" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D18" s="27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E18" s="28"/>
       <c r="F18" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G18" s="26"/>
       <c r="H18" s="26"/>
@@ -3503,17 +3553,17 @@
     <row r="19" ht="30" customHeight="1" spans="1:9">
       <c r="A19" s="23"/>
       <c r="B19" s="27" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D19" s="27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E19" s="28"/>
       <c r="F19" s="28" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G19" s="26"/>
       <c r="H19" s="26"/>
@@ -3522,17 +3572,17 @@
     <row r="20" ht="30" customHeight="1" spans="1:9">
       <c r="A20" s="23"/>
       <c r="B20" s="27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D20" s="27" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E20" s="28"/>
       <c r="F20" s="29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G20" s="26"/>
       <c r="H20" s="26"/>
@@ -3541,17 +3591,17 @@
     <row r="21" ht="45" customHeight="1" spans="1:9">
       <c r="A21" s="23"/>
       <c r="B21" s="27" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E21" s="27"/>
       <c r="F21" s="29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G21" s="26"/>
       <c r="H21" s="26"/>
@@ -3560,17 +3610,17 @@
     <row r="22" ht="45" customHeight="1" spans="1:9">
       <c r="A22" s="23"/>
       <c r="B22" s="27" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D22" s="27" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E22" s="27"/>
       <c r="F22" s="29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G22" s="26"/>
       <c r="H22" s="26"/>
@@ -3579,169 +3629,169 @@
     <row r="23" ht="30" spans="1:9">
       <c r="A23" s="23"/>
       <c r="B23" s="27" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D23" s="27" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E23" s="27"/>
       <c r="F23" s="29" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G23" s="26"/>
       <c r="H23" s="26"/>
       <c r="I23" s="26"/>
     </row>
     <row r="24" ht="45" spans="1:9">
-      <c r="A24" s="32"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="27" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D24" s="27" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E24" s="27"/>
       <c r="F24" s="29" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G24" s="26"/>
       <c r="H24" s="26"/>
       <c r="I24" s="26"/>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:9">
-      <c r="A25" s="32"/>
+      <c r="A25" s="23"/>
       <c r="B25" s="27" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E25" s="27"/>
       <c r="F25" s="29" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G25" s="26"/>
       <c r="H25" s="26"/>
       <c r="I25" s="26"/>
     </row>
     <row r="26" ht="30" spans="1:9">
-      <c r="A26" s="32"/>
+      <c r="A26" s="23"/>
       <c r="B26" s="27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C26" s="27" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D26" s="27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E26" s="27"/>
       <c r="F26" s="29" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G26" s="26"/>
       <c r="H26" s="26"/>
       <c r="I26" s="26"/>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:9">
-      <c r="A27" s="32"/>
+      <c r="A27" s="23"/>
       <c r="B27" s="27" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D27" s="27" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E27" s="27"/>
       <c r="F27" s="29" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G27" s="26"/>
       <c r="H27" s="26"/>
       <c r="I27" s="26"/>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:9">
-      <c r="A28" s="32"/>
+      <c r="A28" s="23"/>
       <c r="B28" s="27" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C28" s="27" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D28" s="27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E28" s="27"/>
       <c r="F28" s="29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G28" s="26"/>
       <c r="H28" s="26"/>
       <c r="I28" s="26"/>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:9">
-      <c r="A29" s="32"/>
+      <c r="A29" s="23"/>
       <c r="B29" s="27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D29" s="27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E29" s="27"/>
       <c r="F29" s="29" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G29" s="26"/>
       <c r="H29" s="26"/>
       <c r="I29" s="26"/>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:9">
-      <c r="A30" s="32"/>
+      <c r="A30" s="23"/>
       <c r="B30" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C30" s="27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D30" s="27" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E30" s="27"/>
       <c r="F30" s="29" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G30" s="26"/>
       <c r="H30" s="26"/>
       <c r="I30" s="26"/>
     </row>
     <row r="31" ht="30" spans="1:9">
-      <c r="A31" s="32"/>
+      <c r="A31" s="23"/>
       <c r="B31" s="27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D31" s="27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E31" s="27"/>
       <c r="F31" s="29" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G31" s="26"/>
       <c r="H31" s="26"/>
@@ -3751,7 +3801,7 @@
       <c r="A32" s="23"/>
       <c r="B32" s="27"/>
       <c r="C32" s="33" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D32" s="29"/>
       <c r="E32" s="27"/>
@@ -3761,209 +3811,209 @@
       <c r="I32" s="26"/>
     </row>
     <row r="33" ht="78.75" customHeight="1" spans="1:9">
-      <c r="A33" s="32"/>
+      <c r="A33" s="23"/>
       <c r="B33" s="27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C33" s="27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D33" s="27" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E33" s="27"/>
       <c r="F33" s="28" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G33" s="26"/>
       <c r="H33" s="26"/>
       <c r="I33" s="26"/>
     </row>
     <row r="34" ht="60" customHeight="1" spans="1:9">
-      <c r="A34" s="32"/>
+      <c r="A34" s="23"/>
       <c r="B34" s="27" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C34" s="27" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D34" s="27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E34" s="27"/>
       <c r="F34" s="28" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G34" s="26"/>
       <c r="H34" s="26"/>
       <c r="I34" s="26"/>
     </row>
     <row r="35" ht="45" customHeight="1" spans="1:9">
-      <c r="A35" s="32"/>
+      <c r="A35" s="23"/>
       <c r="B35" s="27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C35" s="27" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D35" s="27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E35" s="27"/>
       <c r="F35" s="29" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G35" s="26"/>
       <c r="H35" s="26"/>
       <c r="I35" s="26"/>
     </row>
     <row r="36" ht="60" customHeight="1" spans="1:9">
-      <c r="A36" s="32"/>
+      <c r="A36" s="23"/>
       <c r="B36" s="27" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C36" s="27" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D36" s="27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E36" s="27"/>
       <c r="F36" s="28" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G36" s="26"/>
       <c r="H36" s="26"/>
       <c r="I36" s="26"/>
     </row>
     <row r="37" ht="30" spans="1:9">
-      <c r="A37" s="32"/>
+      <c r="A37" s="23"/>
       <c r="B37" s="27" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C37" s="27" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D37" s="27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E37" s="27"/>
       <c r="F37" s="29" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G37" s="26"/>
       <c r="H37" s="26"/>
       <c r="I37" s="26"/>
     </row>
     <row r="38" ht="30" customHeight="1" spans="1:9">
-      <c r="A38" s="32"/>
+      <c r="A38" s="23"/>
       <c r="B38" s="27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C38" s="27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D38" s="27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E38" s="27"/>
       <c r="F38" s="29" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G38" s="26"/>
       <c r="H38" s="26"/>
       <c r="I38" s="26"/>
     </row>
     <row r="39" ht="30" customHeight="1" spans="1:9">
-      <c r="A39" s="32"/>
+      <c r="A39" s="23"/>
       <c r="B39" s="27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C39" s="27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D39" s="27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E39" s="27"/>
       <c r="F39" s="29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G39" s="26"/>
       <c r="H39" s="26"/>
       <c r="I39" s="26"/>
     </row>
     <row r="40" ht="30" customHeight="1" spans="1:9">
-      <c r="A40" s="32"/>
+      <c r="A40" s="23"/>
       <c r="B40" s="27" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C40" s="27" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D40" s="27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E40" s="27"/>
       <c r="F40" s="29" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G40" s="26"/>
       <c r="H40" s="26"/>
       <c r="I40" s="26"/>
     </row>
     <row r="41" ht="30" customHeight="1" spans="1:9">
-      <c r="A41" s="32"/>
+      <c r="A41" s="23"/>
       <c r="B41" s="27" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C41" s="27" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D41" s="27" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E41" s="27"/>
       <c r="F41" s="29" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G41" s="26"/>
       <c r="H41" s="26"/>
       <c r="I41" s="26"/>
     </row>
     <row r="42" ht="30" customHeight="1" spans="1:9">
-      <c r="A42" s="32"/>
+      <c r="A42" s="23"/>
       <c r="B42" s="27" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C42" s="27" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D42" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E42" s="27"/>
       <c r="F42" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G42" s="26"/>
       <c r="H42" s="26"/>
       <c r="I42" s="26"/>
     </row>
     <row r="43" ht="45" customHeight="1" spans="1:9">
-      <c r="A43" s="32"/>
+      <c r="A43" s="23"/>
       <c r="B43" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C43" s="27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D43" s="27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E43" s="27"/>
       <c r="F43" s="27" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G43" s="26"/>
       <c r="H43" s="26"/>
@@ -3984,7 +4034,7 @@
       <c r="A45" s="23"/>
       <c r="B45" s="27"/>
       <c r="C45" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D45" s="29"/>
       <c r="E45" s="27"/>
@@ -3994,133 +4044,133 @@
       <c r="I45" s="26"/>
     </row>
     <row r="46" ht="45" customHeight="1" spans="1:9">
-      <c r="A46" s="32"/>
+      <c r="A46" s="23"/>
       <c r="B46" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D46" s="27" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E46" s="27"/>
       <c r="F46" s="29" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G46" s="26"/>
       <c r="H46" s="26"/>
       <c r="I46" s="26"/>
     </row>
     <row r="47" ht="60" customHeight="1" spans="1:9">
-      <c r="A47" s="32"/>
+      <c r="A47" s="23"/>
       <c r="B47" s="27" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C47" s="27" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D47" s="27" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E47" s="27"/>
       <c r="F47" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G47" s="26"/>
       <c r="H47" s="26"/>
       <c r="I47" s="26"/>
     </row>
     <row r="48" ht="45" customHeight="1" spans="1:9">
-      <c r="A48" s="32"/>
+      <c r="A48" s="23"/>
       <c r="B48" s="27" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D48" s="27" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E48" s="27"/>
       <c r="F48" s="29" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G48" s="26"/>
       <c r="H48" s="26"/>
       <c r="I48" s="26"/>
     </row>
     <row r="49" ht="47.25" customHeight="1" spans="1:9">
-      <c r="A49" s="32"/>
+      <c r="A49" s="23"/>
       <c r="B49" s="27" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C49" s="27" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D49" s="27" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E49" s="27"/>
       <c r="F49" s="28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G49" s="26"/>
       <c r="H49" s="26"/>
       <c r="I49" s="26"/>
     </row>
     <row r="50" ht="45" customHeight="1" spans="1:9">
-      <c r="A50" s="32"/>
+      <c r="A50" s="23"/>
       <c r="B50" s="27" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D50" s="27" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E50" s="27"/>
       <c r="F50" s="29" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G50" s="26"/>
       <c r="H50" s="26"/>
       <c r="I50" s="26"/>
     </row>
     <row r="51" ht="90" customHeight="1" spans="1:9">
-      <c r="A51" s="32"/>
+      <c r="A51" s="23"/>
       <c r="B51" s="27" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D51" s="27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E51" s="27"/>
       <c r="F51" s="29" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G51" s="26"/>
       <c r="H51" s="26"/>
       <c r="I51" s="26"/>
     </row>
     <row r="52" ht="75" customHeight="1" spans="1:9">
-      <c r="A52" s="32"/>
+      <c r="A52" s="23"/>
       <c r="B52" s="27" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C52" s="27" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D52" s="27" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E52" s="27"/>
       <c r="F52" s="29" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G52" s="26"/>
       <c r="H52" s="26"/>
@@ -4130,7 +4180,7 @@
       <c r="A53" s="23"/>
       <c r="B53" s="27"/>
       <c r="C53" s="33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D53" s="29"/>
       <c r="E53" s="27"/>
@@ -4140,114 +4190,114 @@
       <c r="I53" s="26"/>
     </row>
     <row r="54" ht="32.4" customHeight="1" spans="1:9">
-      <c r="A54" s="32"/>
+      <c r="A54" s="23"/>
       <c r="B54" s="27" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C54" s="34" t="s">
-        <v>171</v>
-      </c>
-      <c r="D54" s="31" t="s">
         <v>172</v>
+      </c>
+      <c r="D54" s="32" t="s">
+        <v>173</v>
       </c>
       <c r="E54" s="27"/>
       <c r="F54" s="29" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G54" s="26"/>
       <c r="H54" s="26"/>
       <c r="I54" s="26"/>
     </row>
     <row r="55" ht="31.2" customHeight="1" spans="1:9">
-      <c r="A55" s="32"/>
+      <c r="A55" s="23"/>
       <c r="B55" s="27" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C55" s="34" t="s">
-        <v>175</v>
-      </c>
-      <c r="D55" s="31" t="s">
         <v>176</v>
+      </c>
+      <c r="D55" s="32" t="s">
+        <v>177</v>
       </c>
       <c r="E55" s="27"/>
       <c r="F55" s="29" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G55" s="26"/>
       <c r="H55" s="26"/>
       <c r="I55" s="26"/>
     </row>
     <row r="56" ht="20.4" customHeight="1" spans="1:9">
-      <c r="A56" s="32"/>
+      <c r="A56" s="23"/>
       <c r="B56" s="27" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C56" s="34" t="s">
-        <v>179</v>
-      </c>
-      <c r="D56" s="31" t="s">
         <v>180</v>
+      </c>
+      <c r="D56" s="32" t="s">
+        <v>181</v>
       </c>
       <c r="E56" s="27"/>
       <c r="F56" s="29" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G56" s="26"/>
       <c r="H56" s="26"/>
       <c r="I56" s="26"/>
     </row>
     <row r="57" ht="87" customHeight="1" spans="1:9">
-      <c r="A57" s="32"/>
+      <c r="A57" s="23"/>
       <c r="B57" s="27" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C57" s="34" t="s">
-        <v>183</v>
-      </c>
-      <c r="D57" s="31" t="s">
         <v>184</v>
+      </c>
+      <c r="D57" s="32" t="s">
+        <v>185</v>
       </c>
       <c r="E57" s="27"/>
       <c r="F57" s="28" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G57" s="26"/>
       <c r="H57" s="26"/>
       <c r="I57" s="26"/>
     </row>
     <row r="58" ht="28.8" customHeight="1" spans="1:9">
-      <c r="A58" s="32"/>
+      <c r="A58" s="23"/>
       <c r="B58" s="27" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C58" s="34" t="s">
-        <v>187</v>
-      </c>
-      <c r="D58" s="31" t="s">
         <v>188</v>
+      </c>
+      <c r="D58" s="32" t="s">
+        <v>189</v>
       </c>
       <c r="E58" s="27"/>
       <c r="F58" s="29" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G58" s="26"/>
       <c r="H58" s="26"/>
       <c r="I58" s="26"/>
     </row>
     <row r="59" ht="75" customHeight="1" spans="1:9">
-      <c r="A59" s="32"/>
+      <c r="A59" s="23"/>
       <c r="B59" s="27" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C59" s="34" t="s">
-        <v>191</v>
-      </c>
-      <c r="D59" s="31" t="s">
         <v>192</v>
+      </c>
+      <c r="D59" s="32" t="s">
+        <v>193</v>
       </c>
       <c r="E59" s="27"/>
       <c r="F59" s="29" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G59" s="26"/>
       <c r="H59" s="26"/>
@@ -4257,7 +4307,7 @@
       <c r="A60" s="23"/>
       <c r="B60" s="27"/>
       <c r="C60" s="35" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D60" s="29"/>
       <c r="E60" s="27"/>
@@ -4267,247 +4317,247 @@
       <c r="I60" s="26"/>
     </row>
     <row r="61" ht="28.8" customHeight="1" spans="1:9">
-      <c r="A61" s="32"/>
+      <c r="A61" s="23"/>
       <c r="B61" s="27" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C61" s="27" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D61" s="27" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E61" s="27"/>
       <c r="F61" s="29" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G61" s="26"/>
       <c r="H61" s="26"/>
       <c r="I61" s="26"/>
     </row>
     <row r="62" ht="90" customHeight="1" spans="1:9">
-      <c r="A62" s="32"/>
+      <c r="A62" s="23"/>
       <c r="B62" s="27" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C62" s="27" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D62" s="27" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E62" s="27"/>
       <c r="F62" s="29" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G62" s="26"/>
       <c r="H62" s="26"/>
       <c r="I62" s="26"/>
     </row>
     <row r="63" ht="60" customHeight="1" spans="1:9">
-      <c r="A63" s="32"/>
+      <c r="A63" s="23"/>
       <c r="B63" s="27" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C63" s="27" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D63" s="27" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E63" s="27"/>
       <c r="F63" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G63" s="26"/>
       <c r="H63" s="26"/>
       <c r="I63" s="26"/>
     </row>
     <row r="64" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A64" s="32"/>
+      <c r="A64" s="23"/>
       <c r="B64" s="27" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C64" s="27" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D64" s="27" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E64" s="27"/>
       <c r="F64" s="29" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G64" s="26"/>
       <c r="H64" s="26"/>
       <c r="I64" s="26"/>
     </row>
     <row r="65" ht="45" customHeight="1" spans="1:9">
-      <c r="A65" s="32"/>
+      <c r="A65" s="23"/>
       <c r="B65" s="27" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C65" s="27" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D65" s="27" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E65" s="27"/>
       <c r="F65" s="29" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G65" s="26"/>
       <c r="H65" s="26"/>
       <c r="I65" s="26"/>
     </row>
     <row r="66" ht="30" customHeight="1" spans="1:9">
-      <c r="A66" s="32"/>
+      <c r="A66" s="23"/>
       <c r="B66" s="27" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C66" s="27" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D66" s="27" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E66" s="27"/>
       <c r="F66" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G66" s="26"/>
       <c r="H66" s="26"/>
       <c r="I66" s="26"/>
     </row>
     <row r="67" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A67" s="32"/>
+      <c r="A67" s="23"/>
       <c r="B67" s="27" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C67" s="27" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D67" s="27" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E67" s="27"/>
       <c r="F67" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G67" s="26"/>
       <c r="H67" s="26"/>
       <c r="I67" s="26"/>
     </row>
     <row r="68" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A68" s="32"/>
+      <c r="A68" s="23"/>
       <c r="B68" s="27" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C68" s="27" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D68" s="36" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E68" s="27"/>
       <c r="F68" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G68" s="26"/>
       <c r="H68" s="26"/>
       <c r="I68" s="26"/>
     </row>
     <row r="69" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A69" s="32"/>
+      <c r="A69" s="23"/>
       <c r="B69" s="27" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C69" s="34" t="s">
-        <v>225</v>
-      </c>
-      <c r="D69" s="31" t="s">
         <v>226</v>
+      </c>
+      <c r="D69" s="32" t="s">
+        <v>227</v>
       </c>
       <c r="E69" s="27"/>
       <c r="F69" s="29" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G69" s="26"/>
       <c r="H69" s="26"/>
       <c r="I69" s="26"/>
     </row>
     <row r="70" ht="60" customHeight="1" spans="1:9">
-      <c r="A70" s="32"/>
+      <c r="A70" s="23"/>
       <c r="B70" s="27" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C70" s="27" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D70" s="27" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E70" s="27"/>
       <c r="F70" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G70" s="26"/>
       <c r="H70" s="26"/>
       <c r="I70" s="26"/>
     </row>
     <row r="71" ht="75" customHeight="1" spans="1:9">
-      <c r="A71" s="32"/>
+      <c r="A71" s="23"/>
       <c r="B71" s="27" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C71" s="27" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D71" s="27" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E71" s="27"/>
       <c r="F71" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G71" s="26"/>
       <c r="H71" s="26"/>
       <c r="I71" s="26"/>
     </row>
     <row r="72" ht="45" customHeight="1" spans="1:9">
-      <c r="A72" s="32"/>
+      <c r="A72" s="23"/>
       <c r="B72" s="27" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C72" s="27" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D72" s="27" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E72" s="27"/>
       <c r="F72" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G72" s="26"/>
       <c r="H72" s="26"/>
       <c r="I72" s="26"/>
     </row>
     <row r="73" ht="45" customHeight="1" spans="1:9">
-      <c r="A73" s="32"/>
+      <c r="A73" s="23"/>
       <c r="B73" s="27" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C73" s="27" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D73" s="37" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E73" s="27"/>
       <c r="F73" s="29" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G73" s="26"/>
       <c r="H73" s="26"/>
@@ -4517,7 +4567,7 @@
       <c r="A74" s="23"/>
       <c r="B74" s="27"/>
       <c r="C74" s="38" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D74" s="29"/>
       <c r="E74" s="27"/>
@@ -4527,48 +4577,48 @@
       <c r="I74" s="26"/>
     </row>
     <row r="75" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A75" s="32"/>
+      <c r="A75" s="23"/>
       <c r="B75" s="27" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C75" s="34" t="s">
-        <v>243</v>
-      </c>
-      <c r="D75" s="31" t="s">
         <v>244</v>
+      </c>
+      <c r="D75" s="32" t="s">
+        <v>245</v>
       </c>
       <c r="E75" s="27"/>
       <c r="F75" s="29" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G75" s="26"/>
       <c r="H75" s="26"/>
       <c r="I75" s="26"/>
     </row>
     <row r="76" ht="45" customHeight="1" spans="1:9">
-      <c r="A76" s="32"/>
+      <c r="A76" s="23"/>
       <c r="B76" s="27" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C76" s="34" t="s">
-        <v>247</v>
-      </c>
-      <c r="D76" s="31" t="s">
         <v>248</v>
+      </c>
+      <c r="D76" s="32" t="s">
+        <v>249</v>
       </c>
       <c r="E76" s="27"/>
       <c r="F76" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G76" s="26"/>
       <c r="H76" s="26"/>
       <c r="I76" s="26"/>
     </row>
     <row r="77" ht="15.75" customHeight="1" spans="1:9">
-      <c r="A77" s="32"/>
+      <c r="A77" s="23"/>
       <c r="B77" s="27"/>
       <c r="C77" s="38" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D77" s="29"/>
       <c r="E77" s="27"/>
@@ -4578,186 +4628,186 @@
       <c r="I77" s="26"/>
     </row>
     <row r="78" ht="31.5" customHeight="1" spans="1:9">
-      <c r="A78" s="32"/>
+      <c r="A78" s="23"/>
       <c r="B78" s="27" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C78" s="34" t="s">
-        <v>250</v>
-      </c>
-      <c r="D78" s="31" t="s">
         <v>251</v>
+      </c>
+      <c r="D78" s="32" t="s">
+        <v>252</v>
       </c>
       <c r="E78" s="27"/>
       <c r="F78" s="28" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G78" s="26"/>
       <c r="H78" s="26"/>
       <c r="I78" s="26"/>
     </row>
     <row r="79" ht="30" customHeight="1" spans="1:9">
-      <c r="A79" s="32"/>
+      <c r="A79" s="23"/>
       <c r="B79" s="27" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C79" s="34" t="s">
-        <v>254</v>
-      </c>
-      <c r="D79" s="31" t="s">
         <v>255</v>
+      </c>
+      <c r="D79" s="32" t="s">
+        <v>256</v>
       </c>
       <c r="E79" s="27"/>
       <c r="F79" s="29" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G79" s="26"/>
       <c r="H79" s="26"/>
       <c r="I79" s="26"/>
     </row>
     <row r="80" ht="75" customHeight="1" spans="1:9">
-      <c r="A80" s="32"/>
+      <c r="A80" s="23"/>
       <c r="B80" s="27" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C80" s="34" t="s">
-        <v>258</v>
-      </c>
-      <c r="D80" s="31" t="s">
         <v>259</v>
+      </c>
+      <c r="D80" s="32" t="s">
+        <v>260</v>
       </c>
       <c r="E80" s="27"/>
       <c r="F80" s="29" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G80" s="26"/>
       <c r="H80" s="26"/>
       <c r="I80" s="26"/>
     </row>
     <row r="81" ht="60" customHeight="1" spans="1:9">
-      <c r="A81" s="32"/>
+      <c r="A81" s="23"/>
       <c r="B81" s="27" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C81" s="34" t="s">
-        <v>262</v>
-      </c>
-      <c r="D81" s="31" t="s">
         <v>263</v>
+      </c>
+      <c r="D81" s="32" t="s">
+        <v>264</v>
       </c>
       <c r="E81" s="27"/>
       <c r="F81" s="29" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G81" s="26"/>
       <c r="H81" s="26"/>
       <c r="I81" s="26"/>
     </row>
     <row r="82" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A82" s="32"/>
+      <c r="A82" s="23"/>
       <c r="B82" s="27" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C82" s="34" t="s">
-        <v>266</v>
-      </c>
-      <c r="D82" s="31" t="s">
         <v>267</v>
+      </c>
+      <c r="D82" s="32" t="s">
+        <v>268</v>
       </c>
       <c r="E82" s="27"/>
       <c r="F82" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G82" s="26"/>
       <c r="H82" s="26"/>
       <c r="I82" s="26"/>
     </row>
     <row r="83" ht="45" customHeight="1" spans="1:9">
-      <c r="A83" s="32"/>
+      <c r="A83" s="23"/>
       <c r="B83" s="27" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C83" s="34" t="s">
-        <v>269</v>
-      </c>
-      <c r="D83" s="31" t="s">
         <v>270</v>
+      </c>
+      <c r="D83" s="32" t="s">
+        <v>271</v>
       </c>
       <c r="E83" s="27"/>
       <c r="F83" s="29" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G83" s="26"/>
       <c r="H83" s="26"/>
       <c r="I83" s="26"/>
     </row>
     <row r="84" ht="15.75" customHeight="1" spans="1:9">
-      <c r="A84" s="32"/>
+      <c r="A84" s="23"/>
       <c r="B84" s="27"/>
       <c r="C84" s="38" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D84" s="29"/>
       <c r="E84" s="27"/>
       <c r="F84" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G84" s="26"/>
       <c r="H84" s="26"/>
       <c r="I84" s="26"/>
     </row>
     <row r="85" ht="30" customHeight="1" spans="1:9">
-      <c r="A85" s="32"/>
+      <c r="A85" s="23"/>
       <c r="B85" s="27" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C85" s="34" t="s">
-        <v>274</v>
-      </c>
-      <c r="D85" s="31" t="s">
         <v>275</v>
+      </c>
+      <c r="D85" s="32" t="s">
+        <v>276</v>
       </c>
       <c r="E85" s="27"/>
       <c r="F85" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G85" s="26"/>
       <c r="H85" s="26"/>
       <c r="I85" s="26"/>
     </row>
     <row r="86" ht="30" customHeight="1" spans="1:9">
-      <c r="A86" s="32"/>
+      <c r="A86" s="23"/>
       <c r="B86" s="27" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C86" s="34" t="s">
-        <v>277</v>
-      </c>
-      <c r="D86" s="31" t="s">
         <v>278</v>
+      </c>
+      <c r="D86" s="32" t="s">
+        <v>279</v>
       </c>
       <c r="E86" s="27"/>
       <c r="F86" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G86" s="26"/>
       <c r="H86" s="26"/>
       <c r="I86" s="26"/>
     </row>
     <row r="87" ht="30.75" customHeight="1" spans="1:9">
-      <c r="A87" s="32"/>
+      <c r="A87" s="23"/>
       <c r="B87" s="27" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C87" s="34" t="s">
-        <v>280</v>
-      </c>
-      <c r="D87" s="31" t="s">
         <v>281</v>
+      </c>
+      <c r="D87" s="32" t="s">
+        <v>282</v>
       </c>
       <c r="E87" s="27"/>
       <c r="F87" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G87" s="26"/>
       <c r="H87" s="26"/>
@@ -4767,7 +4817,7 @@
       <c r="A88" s="23"/>
       <c r="B88" s="27"/>
       <c r="C88" s="38" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D88" s="38"/>
       <c r="E88" s="27"/>
@@ -4779,17 +4829,17 @@
     <row r="89" ht="63" customHeight="1" spans="1:9">
       <c r="A89" s="39"/>
       <c r="B89" s="40" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C89" s="41" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D89" s="40" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E89" s="40"/>
       <c r="F89" s="40" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G89" s="26"/>
       <c r="H89" s="26"/>
@@ -4798,19 +4848,19 @@
     <row r="90" ht="78.75" customHeight="1" spans="1:9">
       <c r="A90" s="39"/>
       <c r="B90" s="40" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C90" s="41" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D90" s="40" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E90" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F90" s="40" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G90" s="26"/>
       <c r="H90" s="26"/>
@@ -4819,19 +4869,19 @@
     <row r="91" ht="31.5" customHeight="1" spans="1:9">
       <c r="A91" s="39"/>
       <c r="B91" s="40" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C91" s="41" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D91" s="40" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E91" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F91" s="40" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G91" s="26"/>
       <c r="H91" s="26"/>
@@ -4840,19 +4890,19 @@
     <row r="92" ht="47.25" customHeight="1" spans="1:9">
       <c r="A92" s="39"/>
       <c r="B92" s="40" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C92" s="41" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D92" s="40" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E92" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F92" s="40" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G92" s="26"/>
       <c r="H92" s="26"/>
@@ -4861,19 +4911,19 @@
     <row r="93" ht="31.5" customHeight="1" spans="1:9">
       <c r="A93" s="39"/>
       <c r="B93" s="40" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C93" s="41" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D93" s="40" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E93" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F93" s="40" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G93" s="26"/>
       <c r="H93" s="26"/>
@@ -4882,19 +4932,19 @@
     <row r="94" ht="47.25" customHeight="1" spans="1:9">
       <c r="A94" s="39"/>
       <c r="B94" s="40" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C94" s="41" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D94" s="40" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E94" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F94" s="40" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G94" s="26"/>
       <c r="H94" s="26"/>
@@ -4903,19 +4953,19 @@
     <row r="95" ht="47.25" customHeight="1" spans="1:9">
       <c r="A95" s="39"/>
       <c r="B95" s="40" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C95" s="41" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D95" s="40" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E95" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F95" s="40" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G95" s="26"/>
       <c r="H95" s="26"/>
@@ -4924,19 +4974,19 @@
     <row r="96" ht="31.5" customHeight="1" spans="1:9">
       <c r="A96" s="39"/>
       <c r="B96" s="40" t="s">
+        <v>313</v>
+      </c>
+      <c r="C96" s="41" t="s">
+        <v>314</v>
+      </c>
+      <c r="D96" s="40" t="s">
+        <v>315</v>
+      </c>
+      <c r="E96" s="40" t="s">
+        <v>291</v>
+      </c>
+      <c r="F96" s="40" t="s">
         <v>312</v>
-      </c>
-      <c r="C96" s="41" t="s">
-        <v>313</v>
-      </c>
-      <c r="D96" s="40" t="s">
-        <v>314</v>
-      </c>
-      <c r="E96" s="40" t="s">
-        <v>290</v>
-      </c>
-      <c r="F96" s="40" t="s">
-        <v>311</v>
       </c>
       <c r="G96" s="26"/>
       <c r="H96" s="26"/>
@@ -4945,19 +4995,19 @@
     <row r="97" ht="47.25" customHeight="1" spans="1:9">
       <c r="A97" s="39"/>
       <c r="B97" s="40" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C97" s="41" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D97" s="40" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E97" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F97" s="40" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G97" s="26"/>
       <c r="H97" s="26"/>
@@ -4966,19 +5016,19 @@
     <row r="98" ht="63" customHeight="1" spans="1:9">
       <c r="A98" s="39"/>
       <c r="B98" s="40" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C98" s="41" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D98" s="40" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E98" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F98" s="40" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G98" s="26"/>
       <c r="H98" s="26"/>
@@ -4987,19 +5037,19 @@
     <row r="99" ht="94.5" customHeight="1" spans="1:9">
       <c r="A99" s="39"/>
       <c r="B99" s="40" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C99" s="41" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D99" s="40" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E99" s="42" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F99" s="40" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G99" s="26"/>
       <c r="H99" s="26"/>
@@ -5008,19 +5058,19 @@
     <row r="100" ht="31.5" customHeight="1" spans="1:9">
       <c r="A100" s="39"/>
       <c r="B100" s="40" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C100" s="41" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D100" s="40" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E100" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F100" s="40" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G100" s="26"/>
       <c r="H100" s="26"/>
@@ -5029,19 +5079,19 @@
     <row r="101" ht="47.25" customHeight="1" spans="1:9">
       <c r="A101" s="39"/>
       <c r="B101" s="40" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C101" s="41" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D101" s="40" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E101" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F101" s="40" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G101" s="26"/>
       <c r="H101" s="26"/>
@@ -5050,19 +5100,19 @@
     <row r="102" ht="31.5" customHeight="1" spans="1:9">
       <c r="A102" s="39"/>
       <c r="B102" s="40" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C102" s="41" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D102" s="40" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E102" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F102" s="40" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G102" s="26"/>
       <c r="H102" s="26"/>
@@ -5071,19 +5121,19 @@
     <row r="103" ht="63" customHeight="1" spans="1:9">
       <c r="A103" s="39"/>
       <c r="B103" s="40" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C103" s="41" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D103" s="40" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E103" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F103" s="40" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G103" s="26"/>
       <c r="H103" s="26"/>
@@ -5092,19 +5142,19 @@
     <row r="104" ht="31.5" customHeight="1" spans="1:9">
       <c r="A104" s="39"/>
       <c r="B104" s="40" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C104" s="41" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D104" s="40" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E104" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F104" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G104" s="26"/>
       <c r="H104" s="26"/>
@@ -5113,323 +5163,323 @@
     <row r="105" ht="63" customHeight="1" spans="1:9">
       <c r="A105" s="39"/>
       <c r="B105" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C105" s="41" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D105" s="40" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E105" s="40" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F105" s="40" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G105" s="26"/>
       <c r="H105" s="26"/>
       <c r="I105" s="26"/>
     </row>
     <row r="106" ht="47.25" customHeight="1" spans="1:9">
-      <c r="A106" s="43"/>
+      <c r="A106" s="39"/>
       <c r="B106" s="40" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C106" s="41" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D106" s="40" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E106" s="40"/>
       <c r="F106" s="40" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G106" s="26"/>
       <c r="H106" s="26"/>
       <c r="I106" s="26"/>
     </row>
     <row r="107" ht="31.5" customHeight="1" spans="1:9">
-      <c r="A107" s="43"/>
+      <c r="A107" s="39"/>
       <c r="B107" s="40" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C107" s="41" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D107" s="40" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E107" s="40"/>
       <c r="F107" s="40" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G107" s="26"/>
       <c r="H107" s="26"/>
       <c r="I107" s="26"/>
     </row>
     <row r="108" ht="31.5" customHeight="1" spans="1:9">
-      <c r="A108" s="43"/>
+      <c r="A108" s="39"/>
       <c r="B108" s="40" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C108" s="41" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D108" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E108" s="40"/>
       <c r="F108" s="40" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G108" s="26"/>
       <c r="H108" s="26"/>
       <c r="I108" s="26"/>
     </row>
     <row r="109" ht="31.5" customHeight="1" spans="1:9">
-      <c r="A109" s="43"/>
+      <c r="A109" s="39"/>
       <c r="B109" s="40" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C109" s="41" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D109" s="40" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E109" s="40"/>
       <c r="F109" s="40" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G109" s="26"/>
       <c r="H109" s="26"/>
       <c r="I109" s="26"/>
     </row>
     <row r="110" ht="31.5" customHeight="1" spans="1:9">
-      <c r="A110" s="43"/>
+      <c r="A110" s="39"/>
       <c r="B110" s="40" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C110" s="41" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D110" s="40" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E110" s="40"/>
       <c r="F110" s="40" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G110" s="26"/>
       <c r="H110" s="26"/>
       <c r="I110" s="26"/>
     </row>
     <row r="111" ht="47.25" customHeight="1" spans="1:9">
-      <c r="A111" s="43"/>
+      <c r="A111" s="39"/>
       <c r="B111" s="40" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C111" s="41" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D111" s="40" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E111" s="40"/>
       <c r="F111" s="40" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G111" s="26"/>
       <c r="H111" s="26"/>
       <c r="I111" s="26"/>
     </row>
     <row r="112" ht="47.25" customHeight="1" spans="1:9">
-      <c r="A112" s="43"/>
+      <c r="A112" s="39"/>
       <c r="B112" s="40" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C112" s="41" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D112" s="40" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E112" s="40"/>
       <c r="F112" s="40" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G112" s="26"/>
       <c r="H112" s="26"/>
       <c r="I112" s="26"/>
     </row>
     <row r="113" ht="31.5" customHeight="1" spans="1:9">
-      <c r="A113" s="43"/>
+      <c r="A113" s="39"/>
       <c r="B113" s="40" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C113" s="41" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D113" s="40" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E113" s="40"/>
       <c r="F113" s="40" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G113" s="26"/>
       <c r="H113" s="26"/>
       <c r="I113" s="26"/>
     </row>
     <row r="114" ht="31.5" customHeight="1" spans="1:9">
-      <c r="A114" s="43"/>
+      <c r="A114" s="39"/>
       <c r="B114" s="40" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C114" s="41" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D114" s="40" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E114" s="40"/>
       <c r="F114" s="40" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G114" s="26"/>
       <c r="H114" s="26"/>
       <c r="I114" s="26"/>
     </row>
     <row r="115" ht="31.5" customHeight="1" spans="1:9">
-      <c r="A115" s="43"/>
+      <c r="A115" s="39"/>
       <c r="B115" s="40" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C115" s="41" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D115" s="40" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E115" s="40"/>
       <c r="F115" s="40" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G115" s="26"/>
       <c r="H115" s="26"/>
       <c r="I115" s="26"/>
     </row>
     <row r="116" ht="47.25" customHeight="1" spans="1:9">
-      <c r="A116" s="43"/>
+      <c r="A116" s="39"/>
       <c r="B116" s="40" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C116" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D116" s="40" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E116" s="40"/>
       <c r="F116" s="40" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G116" s="26"/>
       <c r="H116" s="26"/>
       <c r="I116" s="26"/>
     </row>
     <row r="117" ht="47.25" customHeight="1" spans="1:9">
-      <c r="A117" s="43"/>
+      <c r="A117" s="39"/>
       <c r="B117" s="40" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C117" s="41" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D117" s="40" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E117" s="40"/>
       <c r="F117" s="40" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G117" s="26"/>
       <c r="H117" s="26"/>
       <c r="I117" s="26"/>
     </row>
     <row r="118" ht="30" spans="1:9">
-      <c r="A118" s="32"/>
+      <c r="A118" s="23"/>
       <c r="B118" s="27" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C118" s="34" t="s">
-        <v>399</v>
-      </c>
-      <c r="D118" s="31" t="s">
         <v>400</v>
+      </c>
+      <c r="D118" s="32" t="s">
+        <v>401</v>
       </c>
       <c r="E118" s="27"/>
       <c r="F118" s="28" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="G118" s="26"/>
       <c r="H118" s="26"/>
       <c r="I118" s="26"/>
     </row>
     <row r="119" ht="30" spans="1:9">
-      <c r="A119" s="32"/>
+      <c r="A119" s="23"/>
       <c r="B119" s="27" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C119" s="27" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D119" s="27" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E119" s="27"/>
       <c r="F119" s="28" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G119" s="26"/>
       <c r="H119" s="26"/>
       <c r="I119" s="26"/>
     </row>
     <row r="120" ht="30" customHeight="1" spans="1:9">
-      <c r="A120" s="32"/>
+      <c r="A120" s="23"/>
       <c r="B120" s="27" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C120" s="27" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D120" s="27" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E120" s="27"/>
       <c r="F120" s="28" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="G120" s="26"/>
       <c r="H120" s="26"/>
       <c r="I120" s="26"/>
     </row>
     <row r="121" ht="30" customHeight="1" spans="1:9">
-      <c r="A121" s="32"/>
+      <c r="A121" s="23"/>
       <c r="B121" s="27" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C121" s="27" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D121" s="27" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E121" s="27"/>
       <c r="F121" s="28" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="G121" s="26"/>
       <c r="H121" s="26"/>
@@ -5437,499 +5487,535 @@
     </row>
     <row r="122" ht="45" spans="1:9">
       <c r="A122" s="23"/>
-      <c r="B122" s="44" t="s">
-        <v>414</v>
-      </c>
-      <c r="C122" s="45" t="s">
+      <c r="B122" s="27" t="s">
         <v>415</v>
       </c>
-      <c r="D122" s="45" t="s">
+      <c r="C122" s="43" t="s">
         <v>416</v>
       </c>
-      <c r="E122" s="44"/>
-      <c r="F122" s="46"/>
+      <c r="D122" s="43" t="s">
+        <v>417</v>
+      </c>
+      <c r="E122" s="27"/>
+      <c r="F122" s="29" t="s">
+        <v>418</v>
+      </c>
       <c r="G122" s="26"/>
       <c r="H122" s="26"/>
       <c r="I122" s="26"/>
     </row>
-    <row r="123" ht="15.75" spans="1:9">
+    <row r="123" spans="1:9">
       <c r="A123" s="23"/>
-      <c r="B123" s="44" t="s">
-        <v>417</v>
-      </c>
-      <c r="C123" s="44" t="s">
-        <v>418</v>
-      </c>
-      <c r="D123" s="44" t="s">
+      <c r="B123" s="27" t="s">
         <v>419</v>
       </c>
-      <c r="E123" s="44"/>
-      <c r="F123" s="46"/>
+      <c r="C123" s="27" t="s">
+        <v>420</v>
+      </c>
+      <c r="D123" s="27" t="s">
+        <v>421</v>
+      </c>
+      <c r="E123" s="27"/>
+      <c r="F123" s="29" t="s">
+        <v>422</v>
+      </c>
       <c r="G123" s="26"/>
       <c r="H123" s="26"/>
       <c r="I123" s="26"/>
     </row>
     <row r="124" ht="45" spans="1:9">
-      <c r="A124" s="32"/>
+      <c r="A124" s="23"/>
       <c r="B124" s="27" t="s">
-        <v>420</v>
-      </c>
-      <c r="C124" s="45" t="s">
-        <v>421</v>
-      </c>
-      <c r="D124" s="45" t="s">
-        <v>422</v>
+        <v>423</v>
+      </c>
+      <c r="C124" s="43" t="s">
+        <v>424</v>
+      </c>
+      <c r="D124" s="43" t="s">
+        <v>425</v>
       </c>
       <c r="E124" s="27"/>
-      <c r="F124" s="28"/>
+      <c r="F124" s="29" t="s">
+        <v>426</v>
+      </c>
       <c r="G124" s="26"/>
       <c r="H124" s="26"/>
       <c r="I124" s="26"/>
     </row>
     <row r="125" ht="60" spans="1:9">
-      <c r="A125" s="47"/>
-      <c r="B125" s="48" t="s">
-        <v>423</v>
-      </c>
-      <c r="C125" s="45" t="s">
-        <v>424</v>
-      </c>
-      <c r="D125" s="45" t="s">
-        <v>425</v>
-      </c>
-      <c r="E125" s="49"/>
-      <c r="F125" s="49"/>
+      <c r="A125" s="44"/>
+      <c r="B125" s="45" t="s">
+        <v>427</v>
+      </c>
+      <c r="C125" s="43" t="s">
+        <v>428</v>
+      </c>
+      <c r="D125" s="43" t="s">
+        <v>429</v>
+      </c>
+      <c r="E125" s="46"/>
+      <c r="F125" s="29" t="s">
+        <v>430</v>
+      </c>
       <c r="G125" s="26"/>
       <c r="H125" s="26"/>
       <c r="I125" s="26"/>
     </row>
     <row r="126" ht="60" spans="1:9">
-      <c r="A126" s="47"/>
-      <c r="B126" s="50" t="s">
-        <v>426</v>
-      </c>
-      <c r="C126" s="45" t="s">
-        <v>427</v>
-      </c>
-      <c r="D126" s="45" t="s">
-        <v>428</v>
-      </c>
-      <c r="E126" s="49"/>
-      <c r="F126" s="49"/>
+      <c r="A126" s="44"/>
+      <c r="B126" s="47" t="s">
+        <v>431</v>
+      </c>
+      <c r="C126" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="D126" s="43" t="s">
+        <v>433</v>
+      </c>
+      <c r="E126" s="46"/>
+      <c r="F126" s="29" t="s">
+        <v>434</v>
+      </c>
       <c r="G126" s="26"/>
       <c r="H126" s="26"/>
       <c r="I126" s="26"/>
     </row>
     <row r="127" ht="45" spans="1:9">
-      <c r="A127" s="47"/>
-      <c r="B127" s="50" t="s">
-        <v>429</v>
-      </c>
-      <c r="C127" s="45" t="s">
-        <v>430</v>
-      </c>
-      <c r="D127" s="45" t="s">
-        <v>431</v>
-      </c>
-      <c r="E127" s="49"/>
-      <c r="F127" s="49"/>
+      <c r="A127" s="44"/>
+      <c r="B127" s="47" t="s">
+        <v>435</v>
+      </c>
+      <c r="C127" s="43" t="s">
+        <v>436</v>
+      </c>
+      <c r="D127" s="43" t="s">
+        <v>437</v>
+      </c>
+      <c r="E127" s="46"/>
+      <c r="F127" s="29" t="s">
+        <v>438</v>
+      </c>
       <c r="G127" s="26"/>
       <c r="H127" s="26"/>
       <c r="I127" s="26"/>
     </row>
     <row r="128" ht="60" spans="1:9">
-      <c r="A128" s="47"/>
-      <c r="B128" s="50" t="s">
-        <v>432</v>
-      </c>
-      <c r="C128" s="45" t="s">
-        <v>433</v>
-      </c>
-      <c r="D128" s="45" t="s">
-        <v>434</v>
-      </c>
-      <c r="E128" s="49"/>
-      <c r="F128" s="49"/>
+      <c r="A128" s="44"/>
+      <c r="B128" s="47" t="s">
+        <v>439</v>
+      </c>
+      <c r="C128" s="43" t="s">
+        <v>440</v>
+      </c>
+      <c r="D128" s="43" t="s">
+        <v>441</v>
+      </c>
+      <c r="E128" s="46"/>
+      <c r="F128" s="29" t="s">
+        <v>442</v>
+      </c>
       <c r="G128" s="26"/>
       <c r="H128" s="26"/>
       <c r="I128" s="26"/>
     </row>
     <row r="129" ht="60" spans="1:9">
-      <c r="A129" s="47"/>
-      <c r="B129" s="50" t="s">
-        <v>435</v>
-      </c>
-      <c r="C129" s="45" t="s">
-        <v>436</v>
-      </c>
-      <c r="D129" s="45" t="s">
-        <v>437</v>
-      </c>
-      <c r="E129" s="49"/>
-      <c r="F129" s="49"/>
+      <c r="A129" s="44"/>
+      <c r="B129" s="47" t="s">
+        <v>443</v>
+      </c>
+      <c r="C129" s="43" t="s">
+        <v>444</v>
+      </c>
+      <c r="D129" s="43" t="s">
+        <v>445</v>
+      </c>
+      <c r="E129" s="46"/>
+      <c r="F129" s="29" t="s">
+        <v>446</v>
+      </c>
       <c r="G129" s="26"/>
       <c r="H129" s="26"/>
       <c r="I129" s="26"/>
     </row>
     <row r="130" ht="60" spans="1:9">
-      <c r="A130" s="47"/>
-      <c r="B130" s="50" t="s">
-        <v>438</v>
-      </c>
-      <c r="C130" s="45" t="s">
-        <v>439</v>
-      </c>
-      <c r="D130" s="45" t="s">
-        <v>440</v>
-      </c>
-      <c r="E130" s="49"/>
-      <c r="F130" s="49"/>
+      <c r="A130" s="44"/>
+      <c r="B130" s="47" t="s">
+        <v>447</v>
+      </c>
+      <c r="C130" s="43" t="s">
+        <v>448</v>
+      </c>
+      <c r="D130" s="43" t="s">
+        <v>449</v>
+      </c>
+      <c r="E130" s="46"/>
+      <c r="F130" s="29" t="s">
+        <v>450</v>
+      </c>
       <c r="G130" s="26"/>
       <c r="H130" s="26"/>
       <c r="I130" s="26"/>
     </row>
     <row r="131" ht="60" spans="1:9">
-      <c r="A131" s="47"/>
-      <c r="B131" s="50" t="s">
-        <v>441</v>
-      </c>
-      <c r="C131" s="45" t="s">
-        <v>442</v>
-      </c>
-      <c r="D131" s="45" t="s">
-        <v>443</v>
-      </c>
-      <c r="E131" s="49"/>
-      <c r="F131" s="49"/>
+      <c r="A131" s="44"/>
+      <c r="B131" s="47" t="s">
+        <v>451</v>
+      </c>
+      <c r="C131" s="43" t="s">
+        <v>452</v>
+      </c>
+      <c r="D131" s="43" t="s">
+        <v>453</v>
+      </c>
+      <c r="E131" s="46"/>
+      <c r="F131" s="29" t="s">
+        <v>454</v>
+      </c>
       <c r="G131" s="26"/>
       <c r="H131" s="26"/>
       <c r="I131" s="26"/>
     </row>
     <row r="132" ht="60" spans="1:9">
-      <c r="A132" s="47"/>
-      <c r="B132" s="50" t="s">
-        <v>444</v>
-      </c>
-      <c r="C132" s="45" t="s">
-        <v>445</v>
-      </c>
-      <c r="D132" s="45" t="s">
-        <v>446</v>
-      </c>
-      <c r="E132" s="49"/>
-      <c r="F132" s="49"/>
+      <c r="A132" s="44"/>
+      <c r="B132" s="47" t="s">
+        <v>455</v>
+      </c>
+      <c r="C132" s="43" t="s">
+        <v>456</v>
+      </c>
+      <c r="D132" s="43" t="s">
+        <v>457</v>
+      </c>
+      <c r="E132" s="46"/>
+      <c r="F132" s="29" t="s">
+        <v>458</v>
+      </c>
       <c r="G132" s="26"/>
       <c r="H132" s="26"/>
       <c r="I132" s="26"/>
     </row>
     <row r="133" ht="45" spans="1:9">
-      <c r="A133" s="47"/>
-      <c r="B133" s="50" t="s">
-        <v>447</v>
-      </c>
-      <c r="C133" s="45" t="s">
-        <v>448</v>
-      </c>
-      <c r="D133" s="45" t="s">
-        <v>449</v>
-      </c>
-      <c r="E133" s="49"/>
-      <c r="F133" s="49"/>
+      <c r="A133" s="44"/>
+      <c r="B133" s="47" t="s">
+        <v>459</v>
+      </c>
+      <c r="C133" s="43" t="s">
+        <v>460</v>
+      </c>
+      <c r="D133" s="43" t="s">
+        <v>461</v>
+      </c>
+      <c r="E133" s="46"/>
+      <c r="F133" s="29" t="s">
+        <v>462</v>
+      </c>
       <c r="G133" s="26"/>
       <c r="H133" s="26"/>
       <c r="I133" s="26"/>
     </row>
     <row r="134" ht="45" spans="1:9">
-      <c r="A134" s="47"/>
-      <c r="B134" s="51" t="s">
-        <v>450</v>
-      </c>
-      <c r="C134" s="45" t="s">
-        <v>451</v>
-      </c>
-      <c r="D134" s="45" t="s">
-        <v>452</v>
-      </c>
-      <c r="E134" s="49"/>
-      <c r="F134" s="49"/>
+      <c r="A134" s="44"/>
+      <c r="B134" s="48" t="s">
+        <v>463</v>
+      </c>
+      <c r="C134" s="43" t="s">
+        <v>464</v>
+      </c>
+      <c r="D134" s="43" t="s">
+        <v>465</v>
+      </c>
+      <c r="E134" s="46"/>
+      <c r="F134" s="29" t="s">
+        <v>466</v>
+      </c>
       <c r="G134" s="26"/>
       <c r="H134" s="26"/>
       <c r="I134" s="26"/>
     </row>
     <row r="135" ht="45" spans="1:9">
-      <c r="A135" s="47"/>
-      <c r="B135" s="51" t="s">
-        <v>453</v>
-      </c>
-      <c r="C135" s="45" t="s">
-        <v>454</v>
-      </c>
-      <c r="D135" s="45" t="s">
-        <v>455</v>
-      </c>
-      <c r="E135" s="49"/>
-      <c r="F135" s="49"/>
+      <c r="A135" s="44"/>
+      <c r="B135" s="48" t="s">
+        <v>467</v>
+      </c>
+      <c r="C135" s="43" t="s">
+        <v>468</v>
+      </c>
+      <c r="D135" s="43" t="s">
+        <v>469</v>
+      </c>
+      <c r="E135" s="46"/>
+      <c r="F135" s="29" t="s">
+        <v>470</v>
+      </c>
       <c r="G135" s="26"/>
       <c r="H135" s="26"/>
       <c r="I135" s="26"/>
     </row>
     <row r="136" ht="45" spans="1:9">
-      <c r="A136" s="47"/>
-      <c r="B136" s="51" t="s">
-        <v>456</v>
-      </c>
-      <c r="C136" s="45" t="s">
-        <v>457</v>
-      </c>
-      <c r="D136" s="45" t="s">
-        <v>458</v>
-      </c>
-      <c r="E136" s="49"/>
-      <c r="F136" s="49"/>
+      <c r="A136" s="44"/>
+      <c r="B136" s="48" t="s">
+        <v>471</v>
+      </c>
+      <c r="C136" s="43" t="s">
+        <v>472</v>
+      </c>
+      <c r="D136" s="43" t="s">
+        <v>473</v>
+      </c>
+      <c r="E136" s="46"/>
+      <c r="F136" s="29" t="s">
+        <v>474</v>
+      </c>
       <c r="G136" s="26"/>
       <c r="H136" s="26"/>
       <c r="I136" s="26"/>
     </row>
     <row r="137" ht="45" spans="1:9">
-      <c r="A137" s="47"/>
-      <c r="B137" s="51" t="s">
-        <v>459</v>
-      </c>
-      <c r="C137" s="45" t="s">
-        <v>460</v>
-      </c>
-      <c r="D137" s="45" t="s">
-        <v>461</v>
-      </c>
-      <c r="E137" s="49"/>
-      <c r="F137" s="49"/>
+      <c r="A137" s="44"/>
+      <c r="B137" s="48" t="s">
+        <v>475</v>
+      </c>
+      <c r="C137" s="43" t="s">
+        <v>476</v>
+      </c>
+      <c r="D137" s="43" t="s">
+        <v>477</v>
+      </c>
+      <c r="E137" s="46"/>
+      <c r="F137" s="29" t="s">
+        <v>478</v>
+      </c>
       <c r="G137" s="26"/>
       <c r="H137" s="26"/>
       <c r="I137" s="26"/>
     </row>
     <row r="138" ht="45" spans="1:9">
-      <c r="A138" s="47"/>
-      <c r="B138" s="51" t="s">
-        <v>462</v>
-      </c>
-      <c r="C138" s="45" t="s">
-        <v>463</v>
-      </c>
-      <c r="D138" s="45" t="s">
-        <v>464</v>
-      </c>
-      <c r="E138" s="49"/>
-      <c r="F138" s="49"/>
+      <c r="A138" s="44"/>
+      <c r="B138" s="48" t="s">
+        <v>479</v>
+      </c>
+      <c r="C138" s="43" t="s">
+        <v>480</v>
+      </c>
+      <c r="D138" s="43" t="s">
+        <v>481</v>
+      </c>
+      <c r="E138" s="46"/>
+      <c r="F138" s="29" t="s">
+        <v>482</v>
+      </c>
       <c r="G138" s="26"/>
       <c r="H138" s="26"/>
       <c r="I138" s="26"/>
     </row>
     <row r="139" ht="45" spans="1:9">
-      <c r="A139" s="47"/>
-      <c r="B139" s="51" t="s">
-        <v>465</v>
-      </c>
-      <c r="C139" s="45" t="s">
-        <v>466</v>
-      </c>
-      <c r="D139" s="45" t="s">
-        <v>467</v>
-      </c>
-      <c r="E139" s="49"/>
-      <c r="F139" s="49"/>
+      <c r="A139" s="44"/>
+      <c r="B139" s="48" t="s">
+        <v>483</v>
+      </c>
+      <c r="C139" s="43" t="s">
+        <v>484</v>
+      </c>
+      <c r="D139" s="43" t="s">
+        <v>485</v>
+      </c>
+      <c r="E139" s="46"/>
+      <c r="F139" s="29" t="s">
+        <v>486</v>
+      </c>
       <c r="G139" s="26"/>
       <c r="H139" s="26"/>
       <c r="I139" s="26"/>
     </row>
     <row r="140" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A140" s="47"/>
-      <c r="B140" s="47"/>
-      <c r="C140" s="47"/>
-      <c r="D140" s="47"/>
-      <c r="E140" s="47"/>
-      <c r="F140" s="47"/>
+      <c r="A140" s="44"/>
+      <c r="B140" s="44"/>
+      <c r="C140" s="44"/>
+      <c r="D140" s="44"/>
+      <c r="E140" s="44"/>
+      <c r="F140" s="44"/>
       <c r="G140" s="26"/>
       <c r="H140" s="26"/>
       <c r="I140" s="26"/>
     </row>
     <row r="141" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A141" s="47"/>
-      <c r="B141" s="47"/>
-      <c r="C141" s="47"/>
-      <c r="D141" s="47"/>
-      <c r="E141" s="47"/>
-      <c r="F141" s="47"/>
+      <c r="A141" s="44"/>
+      <c r="B141" s="44"/>
+      <c r="C141" s="44"/>
+      <c r="D141" s="44"/>
+      <c r="E141" s="44"/>
+      <c r="F141" s="44"/>
       <c r="G141" s="26"/>
       <c r="H141" s="26"/>
       <c r="I141" s="26"/>
     </row>
     <row r="142" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A142" s="47"/>
-      <c r="B142" s="47"/>
-      <c r="C142" s="47"/>
-      <c r="D142" s="47"/>
-      <c r="E142" s="47"/>
-      <c r="F142" s="47"/>
+      <c r="A142" s="44"/>
+      <c r="B142" s="44"/>
+      <c r="C142" s="44"/>
+      <c r="D142" s="44"/>
+      <c r="E142" s="44"/>
+      <c r="F142" s="44"/>
       <c r="G142" s="26"/>
       <c r="H142" s="26"/>
       <c r="I142" s="26"/>
     </row>
     <row r="143" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A143" s="47"/>
-      <c r="B143" s="47"/>
-      <c r="C143" s="47"/>
-      <c r="D143" s="47"/>
-      <c r="E143" s="47"/>
-      <c r="F143" s="47"/>
+      <c r="A143" s="44"/>
+      <c r="B143" s="44"/>
+      <c r="C143" s="44"/>
+      <c r="D143" s="44"/>
+      <c r="E143" s="44"/>
+      <c r="F143" s="44"/>
       <c r="G143" s="26"/>
       <c r="H143" s="26"/>
       <c r="I143" s="26"/>
     </row>
     <row r="144" ht="14.4" customHeight="1" spans="1:9">
-      <c r="A144" s="52"/>
-      <c r="B144" s="52"/>
-      <c r="C144" s="52"/>
-      <c r="D144" s="52"/>
-      <c r="E144" s="52"/>
-      <c r="F144" s="52"/>
+      <c r="A144" s="49"/>
+      <c r="B144" s="49"/>
+      <c r="C144" s="49"/>
+      <c r="D144" s="49"/>
+      <c r="E144" s="49"/>
+      <c r="F144" s="49"/>
       <c r="G144" s="26"/>
       <c r="H144" s="26"/>
       <c r="I144" s="26"/>
     </row>
     <row r="145" ht="14.4" customHeight="1" spans="1:10">
-      <c r="A145" s="52"/>
-      <c r="B145" s="52"/>
-      <c r="C145" s="52"/>
-      <c r="D145" s="52"/>
-      <c r="E145" s="52"/>
-      <c r="F145" s="52"/>
+      <c r="A145" s="49"/>
+      <c r="B145" s="49"/>
+      <c r="C145" s="49"/>
+      <c r="D145" s="49"/>
+      <c r="E145" s="49"/>
+      <c r="F145" s="49"/>
       <c r="G145" s="26"/>
       <c r="H145" s="26"/>
       <c r="I145" s="26"/>
     </row>
     <row r="146" ht="14.4" customHeight="1" spans="1:10">
-      <c r="A146" s="53" t="s">
-        <v>468</v>
-      </c>
-      <c r="B146" s="54"/>
-      <c r="C146" s="54"/>
-      <c r="D146" s="54"/>
-      <c r="E146" s="54"/>
-      <c r="F146" s="55"/>
+      <c r="A146" s="50" t="s">
+        <v>487</v>
+      </c>
+      <c r="B146" s="51"/>
+      <c r="C146" s="51"/>
+      <c r="D146" s="51"/>
+      <c r="E146" s="51"/>
+      <c r="F146" s="52"/>
       <c r="G146" s="26"/>
       <c r="H146" s="26"/>
       <c r="I146" s="26"/>
     </row>
     <row r="147" ht="16.5" customHeight="1" spans="1:10">
-      <c r="A147" s="56" t="s">
-        <v>469</v>
-      </c>
-      <c r="B147" s="57" t="s">
-        <v>470</v>
-      </c>
-      <c r="C147" s="57" t="s">
-        <v>471</v>
-      </c>
-      <c r="D147" s="58" t="s">
+      <c r="A147" s="53" t="s">
+        <v>488</v>
+      </c>
+      <c r="B147" s="54" t="s">
+        <v>489</v>
+      </c>
+      <c r="C147" s="54" t="s">
+        <v>490</v>
+      </c>
+      <c r="D147" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="E147" s="58" t="s">
-        <v>472</v>
-      </c>
-      <c r="F147" s="59" t="s">
-        <v>473</v>
+      <c r="E147" s="55" t="s">
+        <v>491</v>
+      </c>
+      <c r="F147" s="56" t="s">
+        <v>492</v>
       </c>
       <c r="G147" s="26"/>
       <c r="H147" s="26"/>
       <c r="I147" s="26"/>
     </row>
     <row r="148" ht="15.75" customHeight="1" spans="1:10">
-      <c r="A148" s="60">
+      <c r="A148" s="57">
         <v>1</v>
       </c>
-      <c r="B148" s="61">
+      <c r="B148" s="58">
         <v>43952</v>
       </c>
-      <c r="C148" s="62" t="s">
-        <v>474</v>
-      </c>
-      <c r="D148" s="63" t="s">
-        <v>475</v>
-      </c>
-      <c r="E148" s="64" t="s">
-        <v>476</v>
-      </c>
-      <c r="F148" s="65" t="s">
-        <v>477</v>
+      <c r="C148" s="59" t="s">
+        <v>493</v>
+      </c>
+      <c r="D148" s="60" t="s">
+        <v>494</v>
+      </c>
+      <c r="E148" s="61" t="s">
+        <v>495</v>
+      </c>
+      <c r="F148" s="62" t="s">
+        <v>496</v>
       </c>
       <c r="G148" s="26"/>
       <c r="H148" s="26"/>
       <c r="I148" s="26"/>
     </row>
     <row r="149" ht="31.5" customHeight="1" spans="1:10">
-      <c r="A149" s="66">
+      <c r="A149" s="63">
         <v>2</v>
       </c>
-      <c r="B149" s="67">
+      <c r="B149" s="64">
         <v>44256</v>
       </c>
-      <c r="C149" s="68" t="s">
-        <v>478</v>
-      </c>
-      <c r="D149" s="69" t="s">
-        <v>479</v>
-      </c>
-      <c r="E149" s="68" t="s">
-        <v>476</v>
-      </c>
-      <c r="F149" s="68" t="s">
-        <v>477</v>
+      <c r="C149" s="65" t="s">
+        <v>497</v>
+      </c>
+      <c r="D149" s="66" t="s">
+        <v>498</v>
+      </c>
+      <c r="E149" s="65" t="s">
+        <v>495</v>
+      </c>
+      <c r="F149" s="65" t="s">
+        <v>496</v>
       </c>
       <c r="G149" s="26"/>
       <c r="H149" s="26"/>
       <c r="I149" s="26"/>
     </row>
     <row r="150" ht="44.4" customHeight="1" spans="1:10">
-      <c r="A150" s="70">
+      <c r="A150" s="67">
         <v>3</v>
       </c>
-      <c r="B150" s="71">
+      <c r="B150" s="68">
         <v>44452</v>
       </c>
-      <c r="C150" s="72" t="s">
-        <v>480</v>
-      </c>
-      <c r="D150" s="73" t="s">
-        <v>481</v>
-      </c>
-      <c r="E150" s="72" t="s">
-        <v>476</v>
-      </c>
-      <c r="F150" s="74" t="s">
-        <v>477</v>
+      <c r="C150" s="69" t="s">
+        <v>499</v>
+      </c>
+      <c r="D150" s="70" t="s">
+        <v>500</v>
+      </c>
+      <c r="E150" s="69" t="s">
+        <v>495</v>
+      </c>
+      <c r="F150" s="71" t="s">
+        <v>496</v>
       </c>
       <c r="H150" s="26"/>
       <c r="I150" s="26"/>
       <c r="J150" s="26"/>
     </row>
     <row r="151" ht="16.5" customHeight="1" spans="1:10">
-      <c r="A151" s="75">
+      <c r="A151" s="72">
         <v>4</v>
       </c>
-      <c r="B151" s="76">
+      <c r="B151" s="73">
         <v>46225</v>
       </c>
-      <c r="C151" s="77" t="s">
-        <v>482</v>
-      </c>
-      <c r="D151" s="78" t="s">
-        <v>483</v>
-      </c>
-      <c r="E151" s="77" t="s">
-        <v>484</v>
-      </c>
-      <c r="F151" s="77" t="s">
-        <v>477</v>
+      <c r="C151" s="74" t="s">
+        <v>501</v>
+      </c>
+      <c r="D151" s="75" t="s">
+        <v>502</v>
+      </c>
+      <c r="E151" s="74" t="s">
+        <v>503</v>
+      </c>
+      <c r="F151" s="74" t="s">
+        <v>496</v>
       </c>
       <c r="G151" s="26"/>
       <c r="H151" s="26"/>

</xml_diff>